<commit_message>
cbr: accept both cbr_bop_est row label sets and 15.10.2026 vintage
</commit_message>
<xml_diff>
--- a/cbr/testdata/bop_est.xlsx
+++ b/cbr/testdata/bop_est.xlsx
@@ -9,10 +9,10 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="30690" windowHeight="11505"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="38400" windowHeight="17400"/>
   </bookViews>
   <sheets>
-    <sheet name="Оценка ПБ (14.09.2026)" sheetId="6" r:id="rId1"/>
+    <sheet name="Оценка ПБ (15.10.2026)" sheetId="6" r:id="rId1"/>
   </sheets>
   <externalReferences>
     <externalReference r:id="rId2"/>
@@ -47,25 +47,19 @@
     <definedName name="GPB_IIP_OPTIONS">#REF!</definedName>
     <definedName name="RSQR1">'[4]Reserve pres.'!$E$47</definedName>
     <definedName name="RSQR2">'[4]Reserve pres.'!$E$48</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Оценка ПБ (14.09.2026)'!$A$1:$O$28</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Оценка ПБ (15.10.2026)'!$A$1:$K$28</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="31">
   <si>
     <t>Чистые ошибки и пропуски</t>
   </si>
   <si>
     <t xml:space="preserve">Счет операций с капиталом </t>
-  </si>
-  <si>
-    <t>Доходы к выплате</t>
-  </si>
-  <si>
-    <t>Доходы к получению</t>
   </si>
   <si>
     <t>Импорт</t>
@@ -86,74 +80,24 @@
     <t>Примечание:</t>
   </si>
   <si>
-    <t>Баланс первичных и вторичных доходов</t>
-  </si>
-  <si>
-    <t>Торговый баланс</t>
-  </si>
-  <si>
-    <t>Баланс услуг</t>
-  </si>
-  <si>
     <t>Чистое принятие обязательств</t>
-  </si>
-  <si>
-    <t>Сальдо счета текущих операций и счета операций с капиталом</t>
-  </si>
-  <si>
-    <t>Изменение резервных активов</t>
   </si>
   <si>
     <t>Чистое приобретение финансовых активов, исключая резервные активы</t>
   </si>
   <si>
-    <t>Сальдо финансового счета, исключая резервные активы</t>
-  </si>
-  <si>
     <t>(млрд долларов США)</t>
-  </si>
-  <si>
-    <t>апрель
-2026 г.
-(оценка)</t>
   </si>
   <si>
     <t xml:space="preserve">I квартал 
 2025 г. </t>
   </si>
   <si>
-    <t>апрель
-2025 г.</t>
-  </si>
-  <si>
     <t xml:space="preserve">I квартал 
 2026 г. </t>
   </si>
   <si>
-    <t>май
-2026 г.
-(оценка)</t>
-  </si>
-  <si>
-    <t>май
-2025 г.</t>
-  </si>
-  <si>
-    <t>II квартал 
-2026 г. 
-(оценка)</t>
-  </si>
-  <si>
-    <t>июнь 
-2026 г.
-(оценка)</t>
-  </si>
-  <si>
     <t xml:space="preserve">II квартал 
-2025 г. </t>
-  </si>
-  <si>
-    <t xml:space="preserve">июнь 
 2025 г. </t>
   </si>
   <si>
@@ -161,24 +105,61 @@
 2025 г. </t>
   </si>
   <si>
-    <t>январь - июль
-2025 г.</t>
-  </si>
-  <si>
-    <t>Оценка ключевых агрегатов платежного баланса Российской Федерации за январь - июль 2026 года</t>
-  </si>
-  <si>
     <t>июль 
 2026 г.
 (оценка)</t>
   </si>
   <si>
-    <t>январь - июль 
+    <t>Товары</t>
+  </si>
+  <si>
+    <t>Услуги</t>
+  </si>
+  <si>
+    <t>Первичные и вторичные доходы</t>
+  </si>
+  <si>
+    <t>К получению</t>
+  </si>
+  <si>
+    <t>К выплате</t>
+  </si>
+  <si>
+    <t>Дата последнего обновления: 15 октября 2026 года.</t>
+  </si>
+  <si>
+    <t>Счет текущих операций и счет операций с капиталом</t>
+  </si>
+  <si>
+    <t>Финансовый счет, исключая резервные активы</t>
+  </si>
+  <si>
+    <t>Резервные активы</t>
+  </si>
+  <si>
+    <t>январь - август
 2026 г.
 (оценка)</t>
   </si>
   <si>
-    <t>Дата последнего обновления: 14 сентября 2026 года.</t>
+    <t xml:space="preserve">II квартал 
+2026 г. </t>
+  </si>
+  <si>
+    <t>август
+2026 г.
+(оценка)</t>
+  </si>
+  <si>
+    <t>январь - август
+2025 г.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">август
+2025 г. </t>
+  </si>
+  <si>
+    <t>Оценка ключевых агрегатов платежного баланса Российской Федерации за январь - август 2026 года</t>
   </si>
 </sst>
 </file>
@@ -10468,7 +10449,7 @@
     <xf numFmtId="0" fontId="125" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="125" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="71">
+  <cellXfs count="70">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
@@ -10568,9 +10549,6 @@
     <xf numFmtId="165" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="7" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="4" fontId="4" fillId="0" borderId="22" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="4" fontId="4" fillId="0" borderId="35" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="4" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
@@ -19589,20 +19567,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AJ31"/>
+  <dimension ref="A1:AF31"/>
   <sheetFormatPr defaultColWidth="9.33203125" defaultRowHeight="12.75"/>
   <cols>
     <col min="1" max="1" width="80.5" style="1" customWidth="1"/>
-    <col min="2" max="15" width="13.1640625" style="12" customWidth="1"/>
-    <col min="16" max="17" width="13" style="12" customWidth="1"/>
-    <col min="18" max="18" width="9.33203125" style="1"/>
-    <col min="19" max="19" width="10.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="20" max="16384" width="9.33203125" style="1"/>
+    <col min="2" max="11" width="13.1640625" style="12" customWidth="1"/>
+    <col min="12" max="13" width="13" style="12" customWidth="1"/>
+    <col min="14" max="14" width="9.33203125" style="1"/>
+    <col min="15" max="15" width="10.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="16" max="16384" width="9.33203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" s="3" customFormat="1" ht="18.75">
+    <row r="1" spans="1:32" s="3" customFormat="1" ht="18.75">
       <c r="A1" s="13" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B1" s="6"/>
       <c r="C1" s="6"/>
@@ -19614,391 +19592,317 @@
       <c r="I1" s="6"/>
       <c r="J1" s="6"/>
       <c r="K1" s="6"/>
-      <c r="L1" s="6"/>
-      <c r="M1" s="6"/>
-      <c r="N1" s="6"/>
-      <c r="O1" s="6"/>
-      <c r="P1" s="9"/>
-      <c r="Q1" s="9"/>
-      <c r="R1" s="9"/>
+      <c r="L1" s="9"/>
+      <c r="M1" s="9"/>
+      <c r="N1" s="9"/>
     </row>
-    <row r="2" spans="1:36" s="3" customFormat="1" ht="15.75">
+    <row r="2" spans="1:32" s="3" customFormat="1" ht="15.75">
       <c r="A2" s="32"/>
       <c r="B2" s="6"/>
       <c r="C2" s="6"/>
       <c r="D2" s="6"/>
       <c r="E2" s="6"/>
-      <c r="F2" s="6"/>
+      <c r="F2" s="59"/>
       <c r="G2" s="6"/>
-      <c r="H2" s="60"/>
+      <c r="H2" s="6"/>
       <c r="I2" s="6"/>
       <c r="J2" s="6"/>
-      <c r="K2" s="6"/>
-      <c r="L2" s="6"/>
-      <c r="M2" s="6"/>
-      <c r="N2" s="6"/>
-      <c r="O2" s="9"/>
-      <c r="P2" s="9"/>
-      <c r="Q2" s="9"/>
-      <c r="R2" s="9"/>
+      <c r="K2" s="9"/>
+      <c r="L2" s="9"/>
+      <c r="M2" s="9"/>
+      <c r="N2" s="9"/>
     </row>
-    <row r="3" spans="1:36" s="3" customFormat="1">
-      <c r="L3" s="4"/>
-      <c r="M3" s="4"/>
-      <c r="N3" s="4"/>
-      <c r="O3" s="33" t="s">
-        <v>18</v>
+    <row r="3" spans="1:32" s="3" customFormat="1">
+      <c r="J3" s="4"/>
+      <c r="K3" s="33" t="s">
+        <v>10</v>
       </c>
-      <c r="P3" s="12"/>
+      <c r="L3" s="12"/>
     </row>
-    <row r="4" spans="1:36" s="7" customFormat="1" ht="14.45" customHeight="1">
-      <c r="A4" s="65"/>
-      <c r="B4" s="67" t="s">
-        <v>33</v>
-      </c>
-      <c r="C4" s="61" t="s">
-        <v>22</v>
-      </c>
-      <c r="D4" s="69" t="s">
+    <row r="4" spans="1:32" s="7" customFormat="1" ht="14.45" customHeight="1">
+      <c r="A4" s="64"/>
+      <c r="B4" s="66" t="s">
         <v>25</v>
       </c>
-      <c r="E4" s="63" t="s">
-        <v>19</v>
+      <c r="C4" s="60" t="s">
+        <v>12</v>
       </c>
-      <c r="F4" s="61" t="s">
-        <v>23</v>
-      </c>
-      <c r="G4" s="61" t="s">
+      <c r="D4" s="60" t="s">
         <v>26</v>
       </c>
-      <c r="H4" s="61" t="s">
-        <v>32</v>
+      <c r="E4" s="62" t="s">
+        <v>15</v>
       </c>
-      <c r="I4" s="53" t="s">
-        <v>7</v>
+      <c r="F4" s="68" t="s">
+        <v>27</v>
       </c>
-      <c r="J4" s="54"/>
-      <c r="K4" s="54"/>
-      <c r="L4" s="54"/>
-      <c r="M4" s="54"/>
-      <c r="N4" s="54"/>
-      <c r="O4" s="55"/>
-      <c r="P4" s="9"/>
-      <c r="Q4" s="9"/>
-      <c r="R4" s="9"/>
+      <c r="G4" s="53" t="s">
+        <v>5</v>
+      </c>
+      <c r="H4" s="54"/>
+      <c r="I4" s="54"/>
+      <c r="J4" s="55"/>
+      <c r="K4" s="55"/>
+      <c r="L4" s="9"/>
+      <c r="M4" s="9"/>
+      <c r="N4" s="9"/>
     </row>
-    <row r="5" spans="1:36" s="7" customFormat="1" ht="42.6" customHeight="1">
-      <c r="A5" s="66"/>
-      <c r="B5" s="68"/>
-      <c r="C5" s="62"/>
-      <c r="D5" s="70"/>
-      <c r="E5" s="64"/>
-      <c r="F5" s="62"/>
-      <c r="G5" s="62"/>
-      <c r="H5" s="62"/>
-      <c r="I5" s="58" t="s">
-        <v>30</v>
+    <row r="5" spans="1:32" s="7" customFormat="1" ht="42.6" customHeight="1">
+      <c r="A5" s="65"/>
+      <c r="B5" s="67"/>
+      <c r="C5" s="61"/>
+      <c r="D5" s="61"/>
+      <c r="E5" s="63"/>
+      <c r="F5" s="69"/>
+      <c r="G5" s="58" t="s">
+        <v>28</v>
+      </c>
+      <c r="H5" s="45" t="s">
+        <v>11</v>
+      </c>
+      <c r="I5" s="20" t="s">
+        <v>13</v>
       </c>
       <c r="J5" s="45" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
-      <c r="K5" s="59" t="s">
-        <v>27</v>
+      <c r="K5" s="20" t="s">
+        <v>29</v>
       </c>
-      <c r="L5" s="45" t="s">
+      <c r="L5" s="9"/>
+      <c r="M5" s="9"/>
+      <c r="N5" s="9"/>
+    </row>
+    <row r="6" spans="1:32" ht="15" customHeight="1">
+      <c r="A6" s="22" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" s="17">
+        <v>35</v>
+      </c>
+      <c r="C6" s="47">
+        <v>13.2</v>
+      </c>
+      <c r="D6" s="17">
+        <v>16.899999999999999</v>
+      </c>
+      <c r="E6" s="52">
+        <v>1.6</v>
+      </c>
+      <c r="F6" s="17">
+        <v>3.3</v>
+      </c>
+      <c r="G6" s="40">
         <v>21</v>
       </c>
-      <c r="M5" s="59" t="s">
-        <v>24</v>
-      </c>
-      <c r="N5" s="59" t="s">
-        <v>28</v>
-      </c>
-      <c r="O5" s="20" t="s">
-        <v>29</v>
-      </c>
-      <c r="P5" s="9"/>
-      <c r="Q5" s="9"/>
-      <c r="R5" s="9"/>
-    </row>
-    <row r="6" spans="1:36" ht="15" customHeight="1">
-      <c r="A6" s="22" t="s">
-        <v>6</v>
-      </c>
-      <c r="B6" s="17">
-        <v>33.9</v>
-      </c>
-      <c r="C6" s="47">
-        <v>12.7</v>
-      </c>
-      <c r="D6" s="17">
-        <v>19.5</v>
-      </c>
-      <c r="E6" s="47">
-        <v>6.6</v>
-      </c>
-      <c r="F6" s="52">
-        <v>8.4</v>
-      </c>
-      <c r="G6" s="52">
-        <v>4.5</v>
-      </c>
-      <c r="H6" s="17">
-        <v>1.7</v>
-      </c>
-      <c r="I6" s="40">
-        <v>21.5</v>
-      </c>
-      <c r="J6" s="34">
+      <c r="H6" s="34">
         <v>18.3</v>
       </c>
-      <c r="K6" s="52">
-        <v>2.2000000000000002</v>
+      <c r="I6" s="52">
+        <v>2.1</v>
       </c>
-      <c r="L6" s="46">
-        <v>2.6</v>
-      </c>
-      <c r="M6" s="47">
-        <v>0.9</v>
-      </c>
-      <c r="N6" s="47">
-        <v>-1.3</v>
-      </c>
-      <c r="O6" s="35">
+      <c r="J6" s="46">
         <v>1</v>
       </c>
+      <c r="K6" s="35">
+        <v>-0.5</v>
+      </c>
+      <c r="L6" s="9"/>
+      <c r="M6" s="9"/>
+      <c r="N6" s="9"/>
+      <c r="O6" s="9"/>
       <c r="P6" s="9"/>
       <c r="Q6" s="9"/>
       <c r="R6" s="9"/>
       <c r="S6" s="9"/>
       <c r="T6" s="9"/>
       <c r="U6" s="9"/>
-      <c r="V6" s="9"/>
+      <c r="V6" s="12"/>
       <c r="W6" s="9"/>
       <c r="X6" s="9"/>
       <c r="Y6" s="9"/>
-      <c r="Z6" s="12"/>
+      <c r="Z6" s="9"/>
       <c r="AA6" s="9"/>
       <c r="AB6" s="9"/>
       <c r="AC6" s="9"/>
       <c r="AD6" s="9"/>
       <c r="AE6" s="9"/>
       <c r="AF6" s="9"/>
-      <c r="AG6" s="9"/>
-      <c r="AH6" s="9"/>
-      <c r="AI6" s="9"/>
-      <c r="AJ6" s="9"/>
     </row>
-    <row r="7" spans="1:36">
+    <row r="7" spans="1:32">
       <c r="A7" s="23" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="B7" s="14">
-        <v>79</v>
+        <v>91.6</v>
       </c>
       <c r="C7" s="48">
         <v>27.1</v>
       </c>
       <c r="D7" s="14">
-        <v>38.299999999999997</v>
+        <v>39.4</v>
       </c>
       <c r="E7" s="48">
-        <v>11.6</v>
+        <v>13.3</v>
       </c>
-      <c r="F7" s="48">
-        <v>14.4</v>
+      <c r="F7" s="14">
+        <v>11.7</v>
       </c>
-      <c r="G7" s="48">
-        <v>12.3</v>
+      <c r="G7" s="41">
+        <v>73.3</v>
       </c>
-      <c r="H7" s="14">
-        <v>13.6</v>
+      <c r="H7" s="36">
+        <v>30.6</v>
       </c>
-      <c r="I7" s="41">
-        <v>66</v>
+      <c r="I7" s="48">
+        <v>23.6</v>
       </c>
       <c r="J7" s="36">
-        <v>30.6</v>
-      </c>
-      <c r="K7" s="48">
-        <v>23.6</v>
-      </c>
-      <c r="L7" s="36">
-        <v>8.1</v>
-      </c>
-      <c r="M7" s="48">
-        <v>7.4</v>
-      </c>
-      <c r="N7" s="48">
-        <v>8.1999999999999993</v>
-      </c>
-      <c r="O7" s="14">
         <v>11.8</v>
       </c>
+      <c r="K7" s="14">
+        <v>7.3</v>
+      </c>
+      <c r="L7" s="9"/>
+      <c r="M7" s="9"/>
+      <c r="N7" s="9"/>
+      <c r="O7" s="9"/>
       <c r="P7" s="9"/>
       <c r="Q7" s="9"/>
       <c r="R7" s="9"/>
       <c r="S7" s="9"/>
       <c r="T7" s="9"/>
       <c r="U7" s="9"/>
-      <c r="V7" s="9"/>
+      <c r="V7" s="12"/>
       <c r="W7" s="9"/>
       <c r="X7" s="9"/>
       <c r="Y7" s="9"/>
-      <c r="Z7" s="12"/>
+      <c r="Z7" s="9"/>
       <c r="AA7" s="9"/>
       <c r="AB7" s="9"/>
       <c r="AC7" s="9"/>
       <c r="AD7" s="9"/>
       <c r="AE7" s="9"/>
       <c r="AF7" s="9"/>
-      <c r="AG7" s="9"/>
-      <c r="AH7" s="9"/>
-      <c r="AI7" s="9"/>
-      <c r="AJ7" s="9"/>
     </row>
-    <row r="8" spans="1:36">
+    <row r="8" spans="1:32">
       <c r="A8" s="24" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B8" s="15">
-        <v>271.8</v>
+        <v>312.39999999999998</v>
       </c>
       <c r="C8" s="56">
-        <v>100.7</v>
+        <v>100.9</v>
       </c>
       <c r="D8" s="15">
-        <v>126.1</v>
+        <v>125.7</v>
       </c>
       <c r="E8" s="56">
-        <v>39.6</v>
+        <v>44.8</v>
       </c>
-      <c r="F8" s="56">
-        <v>43.2</v>
+      <c r="F8" s="15">
+        <v>40.9</v>
       </c>
-      <c r="G8" s="56">
-        <v>43.2</v>
+      <c r="G8" s="42">
+        <v>265.7</v>
       </c>
-      <c r="H8" s="15">
-        <v>45</v>
+      <c r="H8" s="37">
+        <v>97.3</v>
       </c>
-      <c r="I8" s="42">
-        <v>233.7</v>
+      <c r="I8" s="49">
+        <v>98.7</v>
       </c>
       <c r="J8" s="37">
-        <v>97.3</v>
-      </c>
-      <c r="K8" s="49">
-        <v>98.7</v>
-      </c>
-      <c r="L8" s="37">
-        <v>33.700000000000003</v>
-      </c>
-      <c r="M8" s="49">
-        <v>32.4</v>
-      </c>
-      <c r="N8" s="49">
-        <v>32.6</v>
-      </c>
-      <c r="O8" s="16">
         <v>37.700000000000003</v>
       </c>
+      <c r="K8" s="16">
+        <v>32</v>
+      </c>
+      <c r="L8" s="9"/>
+      <c r="M8" s="9"/>
+      <c r="N8" s="9"/>
+      <c r="O8" s="9"/>
       <c r="P8" s="9"/>
       <c r="Q8" s="9"/>
       <c r="R8" s="9"/>
       <c r="S8" s="9"/>
       <c r="T8" s="9"/>
       <c r="U8" s="9"/>
-      <c r="V8" s="9"/>
+      <c r="V8" s="12"/>
       <c r="W8" s="9"/>
       <c r="X8" s="9"/>
       <c r="Y8" s="9"/>
-      <c r="Z8" s="12"/>
+      <c r="Z8" s="9"/>
       <c r="AA8" s="9"/>
       <c r="AB8" s="9"/>
       <c r="AC8" s="9"/>
       <c r="AD8" s="9"/>
       <c r="AE8" s="9"/>
       <c r="AF8" s="9"/>
-      <c r="AG8" s="9"/>
-      <c r="AH8" s="9"/>
-      <c r="AI8" s="9"/>
-      <c r="AJ8" s="9"/>
     </row>
-    <row r="9" spans="1:36">
+    <row r="9" spans="1:32">
       <c r="A9" s="25" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B9" s="19">
-        <v>192.8</v>
+        <v>220.8</v>
       </c>
       <c r="C9" s="57">
-        <v>73.599999999999994</v>
+        <v>73.8</v>
       </c>
       <c r="D9" s="19">
-        <v>87.8</v>
+        <v>86.3</v>
       </c>
       <c r="E9" s="57">
-        <v>28</v>
+        <v>31.5</v>
       </c>
-      <c r="F9" s="57">
-        <v>28.8</v>
+      <c r="F9" s="19">
+        <v>29.2</v>
       </c>
-      <c r="G9" s="57">
-        <v>30.9</v>
+      <c r="G9" s="43">
+        <v>192.4</v>
       </c>
-      <c r="H9" s="19">
-        <v>31.4</v>
+      <c r="H9" s="38">
+        <v>66.7</v>
       </c>
-      <c r="I9" s="43">
-        <v>167.7</v>
+      <c r="I9" s="50">
+        <v>75.099999999999994</v>
       </c>
       <c r="J9" s="38">
-        <v>66.7</v>
-      </c>
-      <c r="K9" s="50">
-        <v>75.099999999999994</v>
-      </c>
-      <c r="L9" s="38">
-        <v>25.6</v>
-      </c>
-      <c r="M9" s="50">
-        <v>25</v>
-      </c>
-      <c r="N9" s="50">
-        <v>24.4</v>
-      </c>
-      <c r="O9" s="21">
         <v>25.9</v>
       </c>
+      <c r="K9" s="21">
+        <v>24.8</v>
+      </c>
+      <c r="L9" s="9"/>
+      <c r="M9" s="9"/>
+      <c r="N9" s="9"/>
+      <c r="O9" s="9"/>
       <c r="P9" s="9"/>
       <c r="Q9" s="9"/>
       <c r="R9" s="9"/>
       <c r="S9" s="9"/>
       <c r="T9" s="9"/>
       <c r="U9" s="9"/>
-      <c r="V9" s="9"/>
+      <c r="V9" s="12"/>
       <c r="W9" s="9"/>
       <c r="X9" s="9"/>
       <c r="Y9" s="9"/>
-      <c r="Z9" s="12"/>
+      <c r="Z9" s="9"/>
       <c r="AA9" s="9"/>
       <c r="AB9" s="9"/>
       <c r="AC9" s="9"/>
       <c r="AD9" s="9"/>
       <c r="AE9" s="9"/>
       <c r="AF9" s="9"/>
-      <c r="AG9" s="9"/>
-      <c r="AH9" s="9"/>
-      <c r="AI9" s="9"/>
-      <c r="AJ9" s="9"/>
     </row>
-    <row r="10" spans="1:36" s="10" customFormat="1">
+    <row r="10" spans="1:32" s="10" customFormat="1">
       <c r="A10" s="23" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="B10" s="14">
-        <v>-27.9</v>
+        <v>-33.700000000000003</v>
       </c>
       <c r="C10" s="48">
         <v>-8.8000000000000007</v>
@@ -20007,401 +19911,329 @@
         <v>-13.1</v>
       </c>
       <c r="E10" s="48">
-        <v>-3.2</v>
+        <v>-5.4</v>
       </c>
-      <c r="F10" s="48">
-        <v>-4.3</v>
+      <c r="F10" s="14">
+        <v>-6.3</v>
       </c>
-      <c r="G10" s="48">
-        <v>-5.7</v>
+      <c r="G10" s="41">
+        <v>-31.4</v>
       </c>
-      <c r="H10" s="14">
-        <v>-6</v>
+      <c r="H10" s="36">
+        <v>-7.6</v>
       </c>
-      <c r="I10" s="41">
-        <v>-25.6</v>
+      <c r="I10" s="48">
+        <v>-12.6</v>
       </c>
       <c r="J10" s="36">
-        <v>-7.6</v>
-      </c>
-      <c r="K10" s="48">
-        <v>-12.6</v>
-      </c>
-      <c r="L10" s="36">
-        <v>-3.2</v>
-      </c>
-      <c r="M10" s="48">
-        <v>-4.5999999999999996</v>
-      </c>
-      <c r="N10" s="48">
-        <v>-4.8</v>
-      </c>
-      <c r="O10" s="14">
         <v>-5.4</v>
       </c>
+      <c r="K10" s="14">
+        <v>-5.8</v>
+      </c>
+      <c r="L10" s="9"/>
+      <c r="M10" s="9"/>
+      <c r="N10" s="9"/>
+      <c r="O10" s="9"/>
       <c r="P10" s="9"/>
       <c r="Q10" s="9"/>
       <c r="R10" s="9"/>
       <c r="S10" s="9"/>
       <c r="T10" s="9"/>
       <c r="U10" s="9"/>
-      <c r="V10" s="9"/>
+      <c r="V10" s="12"/>
       <c r="W10" s="9"/>
       <c r="X10" s="9"/>
       <c r="Y10" s="9"/>
-      <c r="Z10" s="12"/>
+      <c r="Z10" s="9"/>
       <c r="AA10" s="9"/>
       <c r="AB10" s="9"/>
       <c r="AC10" s="9"/>
       <c r="AD10" s="9"/>
       <c r="AE10" s="9"/>
       <c r="AF10" s="9"/>
-      <c r="AG10" s="9"/>
-      <c r="AH10" s="9"/>
-      <c r="AI10" s="9"/>
-      <c r="AJ10" s="9"/>
     </row>
-    <row r="11" spans="1:36" s="10" customFormat="1">
+    <row r="11" spans="1:32" s="10" customFormat="1">
       <c r="A11" s="24" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B11" s="15">
-        <v>27.4</v>
+        <v>31.1</v>
       </c>
       <c r="C11" s="56">
         <v>11.3</v>
       </c>
       <c r="D11" s="15">
-        <v>12</v>
+        <v>11.9</v>
       </c>
       <c r="E11" s="56">
-        <v>4</v>
+        <v>4.3</v>
       </c>
-      <c r="F11" s="56">
+      <c r="F11" s="15">
+        <v>3.6</v>
+      </c>
+      <c r="G11" s="42">
+        <v>30.7</v>
+      </c>
+      <c r="H11" s="37">
+        <v>10.3</v>
+      </c>
+      <c r="I11" s="49">
+        <v>12.1</v>
+      </c>
+      <c r="J11" s="37">
+        <v>4.2</v>
+      </c>
+      <c r="K11" s="16">
         <v>4.0999999999999996</v>
       </c>
-      <c r="G11" s="56">
-        <v>4</v>
-      </c>
-      <c r="H11" s="15">
-        <v>4.2</v>
-      </c>
-      <c r="I11" s="42">
-        <v>26.6</v>
-      </c>
-      <c r="J11" s="37">
-        <v>10.3</v>
-      </c>
-      <c r="K11" s="49">
-        <v>12.1</v>
-      </c>
-      <c r="L11" s="37">
-        <v>4.3</v>
-      </c>
-      <c r="M11" s="49">
-        <v>3.8</v>
-      </c>
-      <c r="N11" s="49">
-        <v>4</v>
-      </c>
-      <c r="O11" s="16">
-        <v>4.2</v>
-      </c>
+      <c r="L11" s="9"/>
+      <c r="M11" s="9"/>
+      <c r="N11" s="9"/>
+      <c r="O11" s="9"/>
       <c r="P11" s="9"/>
       <c r="Q11" s="9"/>
       <c r="R11" s="9"/>
       <c r="S11" s="9"/>
       <c r="T11" s="9"/>
       <c r="U11" s="9"/>
-      <c r="V11" s="9"/>
+      <c r="V11" s="12"/>
       <c r="W11" s="9"/>
       <c r="X11" s="9"/>
       <c r="Y11" s="9"/>
-      <c r="Z11" s="12"/>
+      <c r="Z11" s="9"/>
       <c r="AA11" s="9"/>
       <c r="AB11" s="9"/>
       <c r="AC11" s="9"/>
       <c r="AD11" s="9"/>
       <c r="AE11" s="9"/>
       <c r="AF11" s="9"/>
-      <c r="AG11" s="9"/>
-      <c r="AH11" s="9"/>
-      <c r="AI11" s="9"/>
-      <c r="AJ11" s="9"/>
     </row>
-    <row r="12" spans="1:36" s="10" customFormat="1">
+    <row r="12" spans="1:32" s="10" customFormat="1">
       <c r="A12" s="25" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B12" s="19">
-        <v>55.4</v>
+        <v>64.8</v>
       </c>
       <c r="C12" s="57">
         <v>20.100000000000001</v>
       </c>
       <c r="D12" s="19">
-        <v>25.2</v>
+        <v>25.1</v>
       </c>
       <c r="E12" s="57">
-        <v>7.2</v>
-      </c>
-      <c r="F12" s="57">
-        <v>8.3000000000000007</v>
-      </c>
-      <c r="G12" s="57">
         <v>9.6999999999999993</v>
       </c>
-      <c r="H12" s="19">
-        <v>10.1</v>
+      <c r="F12" s="19">
+        <v>9.9</v>
       </c>
-      <c r="I12" s="43">
-        <v>52.2</v>
+      <c r="G12" s="43">
+        <v>62.1</v>
+      </c>
+      <c r="H12" s="38">
+        <v>17.8</v>
+      </c>
+      <c r="I12" s="50">
+        <v>24.7</v>
       </c>
       <c r="J12" s="38">
-        <v>17.8</v>
-      </c>
-      <c r="K12" s="50">
-        <v>24.7</v>
-      </c>
-      <c r="L12" s="38">
-        <v>7.5</v>
-      </c>
-      <c r="M12" s="50">
-        <v>8.4</v>
-      </c>
-      <c r="N12" s="50">
-        <v>8.8000000000000007</v>
-      </c>
-      <c r="O12" s="21">
         <v>9.6999999999999993</v>
       </c>
+      <c r="K12" s="21">
+        <v>9.9</v>
+      </c>
+      <c r="L12" s="9"/>
+      <c r="M12" s="9"/>
+      <c r="N12" s="9"/>
+      <c r="O12" s="9"/>
       <c r="P12" s="9"/>
       <c r="Q12" s="9"/>
       <c r="R12" s="9"/>
       <c r="S12" s="9"/>
       <c r="T12" s="9"/>
       <c r="U12" s="9"/>
-      <c r="V12" s="9"/>
+      <c r="V12" s="12"/>
       <c r="W12" s="9"/>
       <c r="X12" s="9"/>
       <c r="Y12" s="9"/>
-      <c r="Z12" s="12"/>
+      <c r="Z12" s="9"/>
       <c r="AA12" s="9"/>
       <c r="AB12" s="9"/>
       <c r="AC12" s="9"/>
       <c r="AD12" s="9"/>
       <c r="AE12" s="9"/>
       <c r="AF12" s="9"/>
-      <c r="AG12" s="9"/>
-      <c r="AH12" s="9"/>
-      <c r="AI12" s="9"/>
-      <c r="AJ12" s="9"/>
     </row>
-    <row r="13" spans="1:36">
+    <row r="13" spans="1:32">
       <c r="A13" s="23" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="B13" s="14">
-        <v>-17.2</v>
+        <v>-22.9</v>
       </c>
       <c r="C13" s="48">
-        <v>-5.6</v>
+        <v>-5.0999999999999996</v>
       </c>
       <c r="D13" s="14">
-        <v>-5.7</v>
+        <v>-9.3000000000000007</v>
       </c>
       <c r="E13" s="48">
-        <v>-1.8</v>
+        <v>-6.4</v>
       </c>
-      <c r="F13" s="48">
-        <v>-1.7</v>
-      </c>
-      <c r="G13" s="48">
+      <c r="F13" s="14">
         <v>-2.1</v>
       </c>
-      <c r="H13" s="14">
-        <v>-5.9</v>
+      <c r="G13" s="41">
+        <v>-20.9</v>
       </c>
-      <c r="I13" s="41">
-        <v>-18.899999999999999</v>
+      <c r="H13" s="36">
+        <v>-4.7</v>
+      </c>
+      <c r="I13" s="48">
+        <v>-8.9</v>
       </c>
       <c r="J13" s="36">
-        <v>-4.7</v>
-      </c>
-      <c r="K13" s="48">
-        <v>-8.9</v>
-      </c>
-      <c r="L13" s="36">
-        <v>-2.2000000000000002</v>
-      </c>
-      <c r="M13" s="48">
-        <v>-1.9</v>
-      </c>
-      <c r="N13" s="48">
-        <v>-4.7</v>
-      </c>
-      <c r="O13" s="14">
         <v>-5.3</v>
       </c>
+      <c r="K13" s="14">
+        <v>-2</v>
+      </c>
+      <c r="L13" s="9"/>
+      <c r="M13" s="9"/>
+      <c r="N13" s="9"/>
+      <c r="O13" s="9"/>
       <c r="P13" s="9"/>
       <c r="Q13" s="9"/>
       <c r="R13" s="9"/>
       <c r="S13" s="9"/>
       <c r="T13" s="9"/>
       <c r="U13" s="9"/>
-      <c r="V13" s="9"/>
+      <c r="V13" s="12"/>
       <c r="W13" s="9"/>
       <c r="X13" s="9"/>
       <c r="Y13" s="9"/>
-      <c r="Z13" s="12"/>
+      <c r="Z13" s="9"/>
       <c r="AA13" s="9"/>
       <c r="AB13" s="9"/>
       <c r="AC13" s="9"/>
       <c r="AD13" s="9"/>
       <c r="AE13" s="9"/>
       <c r="AF13" s="9"/>
-      <c r="AG13" s="9"/>
-      <c r="AH13" s="9"/>
-      <c r="AI13" s="9"/>
-      <c r="AJ13" s="9"/>
     </row>
-    <row r="14" spans="1:36">
+    <row r="14" spans="1:32">
       <c r="A14" s="24" t="s">
-        <v>3</v>
+        <v>19</v>
       </c>
       <c r="B14" s="16">
-        <v>23.5</v>
+        <v>26.5</v>
       </c>
       <c r="C14" s="49">
-        <v>8.6999999999999993</v>
+        <v>9.1999999999999993</v>
       </c>
       <c r="D14" s="16">
-        <v>10.9</v>
+        <v>10.8</v>
       </c>
       <c r="E14" s="49">
-        <v>3.1</v>
-      </c>
-      <c r="F14" s="49">
         <v>4</v>
       </c>
-      <c r="G14" s="49">
-        <v>3.8</v>
+      <c r="F14" s="16">
+        <v>2.5</v>
       </c>
-      <c r="H14" s="16">
-        <v>3.9</v>
+      <c r="G14" s="42">
+        <v>23.4</v>
       </c>
-      <c r="I14" s="42">
-        <v>20.9</v>
+      <c r="H14" s="37">
+        <v>7.9</v>
+      </c>
+      <c r="I14" s="49">
+        <v>8.9</v>
       </c>
       <c r="J14" s="37">
-        <v>7.9</v>
+        <v>4.0999999999999996</v>
       </c>
-      <c r="K14" s="49">
-        <v>8.9</v>
-      </c>
-      <c r="L14" s="37">
-        <v>3.1</v>
-      </c>
-      <c r="M14" s="49">
+      <c r="K14" s="16">
         <v>2.6</v>
       </c>
-      <c r="N14" s="49">
-        <v>3.3</v>
-      </c>
-      <c r="O14" s="16">
-        <v>4.0999999999999996</v>
-      </c>
+      <c r="L14" s="9"/>
+      <c r="M14" s="9"/>
+      <c r="N14" s="9"/>
+      <c r="O14" s="9"/>
       <c r="P14" s="9"/>
       <c r="Q14" s="9"/>
       <c r="R14" s="9"/>
       <c r="S14" s="9"/>
       <c r="T14" s="9"/>
       <c r="U14" s="9"/>
-      <c r="V14" s="9"/>
+      <c r="V14" s="12"/>
       <c r="W14" s="9"/>
       <c r="X14" s="9"/>
       <c r="Y14" s="9"/>
-      <c r="Z14" s="12"/>
+      <c r="Z14" s="9"/>
       <c r="AA14" s="9"/>
       <c r="AB14" s="9"/>
       <c r="AC14" s="9"/>
       <c r="AD14" s="9"/>
       <c r="AE14" s="9"/>
       <c r="AF14" s="9"/>
-      <c r="AG14" s="9"/>
-      <c r="AH14" s="9"/>
-      <c r="AI14" s="9"/>
-      <c r="AJ14" s="9"/>
     </row>
-    <row r="15" spans="1:36">
+    <row r="15" spans="1:32">
       <c r="A15" s="25" t="s">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="B15" s="21">
-        <v>40.6</v>
+        <v>49.4</v>
       </c>
       <c r="C15" s="50">
-        <v>14.3</v>
+        <v>14.4</v>
       </c>
       <c r="D15" s="21">
-        <v>16.600000000000001</v>
+        <v>20.2</v>
       </c>
       <c r="E15" s="50">
-        <v>5</v>
+        <v>10.3</v>
       </c>
-      <c r="F15" s="50">
-        <v>5.7</v>
+      <c r="F15" s="21">
+        <v>4.5999999999999996</v>
       </c>
-      <c r="G15" s="50">
-        <v>5.9</v>
+      <c r="G15" s="43">
+        <v>44.3</v>
       </c>
-      <c r="H15" s="21">
-        <v>9.8000000000000007</v>
+      <c r="H15" s="38">
+        <v>12.6</v>
       </c>
-      <c r="I15" s="43">
-        <v>39.799999999999997</v>
+      <c r="I15" s="50">
+        <v>17.8</v>
       </c>
       <c r="J15" s="38">
-        <v>12.7</v>
+        <v>9.4</v>
       </c>
-      <c r="K15" s="50">
-        <v>17.8</v>
-      </c>
-      <c r="L15" s="38">
-        <v>5.3</v>
-      </c>
-      <c r="M15" s="50">
+      <c r="K15" s="21">
         <v>4.5</v>
       </c>
-      <c r="N15" s="50">
-        <v>8</v>
-      </c>
-      <c r="O15" s="21">
-        <v>9.4</v>
-      </c>
+      <c r="L15" s="9"/>
+      <c r="M15" s="9"/>
+      <c r="N15" s="9"/>
+      <c r="O15" s="9"/>
       <c r="P15" s="9"/>
       <c r="Q15" s="9"/>
       <c r="R15" s="9"/>
       <c r="S15" s="9"/>
       <c r="T15" s="9"/>
       <c r="U15" s="9"/>
-      <c r="V15" s="9"/>
+      <c r="V15" s="12"/>
       <c r="W15" s="9"/>
       <c r="X15" s="9"/>
       <c r="Y15" s="9"/>
-      <c r="Z15" s="12"/>
+      <c r="Z15" s="9"/>
       <c r="AA15" s="9"/>
       <c r="AB15" s="9"/>
       <c r="AC15" s="9"/>
       <c r="AD15" s="9"/>
       <c r="AE15" s="9"/>
       <c r="AF15" s="9"/>
-      <c r="AG15" s="9"/>
-      <c r="AH15" s="9"/>
-      <c r="AI15" s="9"/>
-      <c r="AJ15" s="9"/>
     </row>
-    <row r="16" spans="1:36" ht="14.25">
+    <row r="16" spans="1:32" ht="14.25">
       <c r="A16" s="26" t="s">
         <v>1</v>
       </c>
@@ -20417,335 +20249,275 @@
       <c r="E16" s="51">
         <v>0</v>
       </c>
-      <c r="F16" s="51">
+      <c r="F16" s="18">
         <v>0</v>
       </c>
-      <c r="G16" s="51">
+      <c r="G16" s="44">
+        <v>-0.2</v>
+      </c>
+      <c r="H16" s="39">
+        <v>-0.1</v>
+      </c>
+      <c r="I16" s="51">
+        <v>-0.1</v>
+      </c>
+      <c r="J16" s="39">
         <v>0</v>
       </c>
-      <c r="H16" s="18">
-        <v>0</v>
-      </c>
-      <c r="I16" s="44">
-        <v>-0.2</v>
-      </c>
-      <c r="J16" s="39">
+      <c r="K16" s="18">
         <v>-0.1</v>
       </c>
-      <c r="K16" s="51">
-        <v>-0.1</v>
-      </c>
-      <c r="L16" s="39">
-        <v>0</v>
-      </c>
-      <c r="M16" s="51">
-        <v>-0.1</v>
-      </c>
-      <c r="N16" s="51">
-        <v>0</v>
-      </c>
-      <c r="O16" s="18">
-        <v>0</v>
-      </c>
+      <c r="L16" s="9"/>
+      <c r="M16" s="9"/>
+      <c r="N16" s="9"/>
+      <c r="O16" s="9"/>
       <c r="P16" s="9"/>
       <c r="Q16" s="9"/>
       <c r="R16" s="9"/>
       <c r="S16" s="9"/>
       <c r="T16" s="9"/>
       <c r="U16" s="9"/>
-      <c r="V16" s="9"/>
+      <c r="V16" s="12"/>
       <c r="W16" s="9"/>
       <c r="X16" s="9"/>
       <c r="Y16" s="9"/>
-      <c r="Z16" s="12"/>
+      <c r="Z16" s="9"/>
       <c r="AA16" s="9"/>
       <c r="AB16" s="9"/>
       <c r="AC16" s="9"/>
       <c r="AD16" s="9"/>
       <c r="AE16" s="9"/>
       <c r="AF16" s="9"/>
-      <c r="AG16" s="9"/>
-      <c r="AH16" s="9"/>
-      <c r="AI16" s="9"/>
-      <c r="AJ16" s="9"/>
     </row>
-    <row r="17" spans="1:36" ht="14.25">
+    <row r="17" spans="1:32" ht="14.25">
       <c r="A17" s="27" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="B17" s="18">
-        <v>33.799999999999997</v>
+        <v>35</v>
       </c>
       <c r="C17" s="51">
-        <v>12.6</v>
+        <v>13.1</v>
       </c>
       <c r="D17" s="18">
-        <v>19.5</v>
+        <v>16.899999999999999</v>
       </c>
       <c r="E17" s="51">
-        <v>6.6</v>
+        <v>1.5</v>
       </c>
-      <c r="F17" s="51">
-        <v>8.4</v>
+      <c r="F17" s="18">
+        <v>3.3</v>
       </c>
-      <c r="G17" s="51">
-        <v>4.5</v>
+      <c r="G17" s="44">
+        <v>20.7</v>
       </c>
-      <c r="H17" s="18">
-        <v>1.7</v>
+      <c r="H17" s="39">
+        <v>18.3</v>
       </c>
-      <c r="I17" s="44">
-        <v>21.3</v>
+      <c r="I17" s="51">
+        <v>2</v>
       </c>
       <c r="J17" s="39">
-        <v>18.2</v>
-      </c>
-      <c r="K17" s="51">
-        <v>2.1</v>
-      </c>
-      <c r="L17" s="39">
-        <v>2.6</v>
-      </c>
-      <c r="M17" s="51">
-        <v>0.8</v>
-      </c>
-      <c r="N17" s="51">
-        <v>-1.3</v>
-      </c>
-      <c r="O17" s="18">
         <v>1</v>
       </c>
+      <c r="K17" s="18">
+        <v>-0.5</v>
+      </c>
+      <c r="L17" s="9"/>
+      <c r="M17" s="9"/>
+      <c r="N17" s="9"/>
+      <c r="O17" s="9"/>
       <c r="P17" s="9"/>
       <c r="Q17" s="9"/>
       <c r="R17" s="9"/>
       <c r="S17" s="9"/>
       <c r="T17" s="9"/>
       <c r="U17" s="9"/>
-      <c r="V17" s="9"/>
+      <c r="V17" s="12"/>
       <c r="W17" s="9"/>
       <c r="X17" s="9"/>
       <c r="Y17" s="9"/>
-      <c r="Z17" s="12"/>
+      <c r="Z17" s="9"/>
       <c r="AA17" s="9"/>
       <c r="AB17" s="9"/>
       <c r="AC17" s="9"/>
       <c r="AD17" s="9"/>
       <c r="AE17" s="9"/>
       <c r="AF17" s="9"/>
-      <c r="AG17" s="9"/>
-      <c r="AH17" s="9"/>
-      <c r="AI17" s="9"/>
-      <c r="AJ17" s="9"/>
     </row>
-    <row r="18" spans="1:36" ht="13.15" customHeight="1">
+    <row r="18" spans="1:32" ht="13.15" customHeight="1">
       <c r="A18" s="28" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="B18" s="17">
-        <v>17.3</v>
+        <v>24</v>
       </c>
       <c r="C18" s="52">
-        <v>17.899999999999999</v>
+        <v>19.100000000000001</v>
       </c>
       <c r="D18" s="17">
-        <v>2.2000000000000002</v>
+        <v>1</v>
       </c>
       <c r="E18" s="52">
-        <v>4.5</v>
+        <v>-2.5</v>
       </c>
-      <c r="F18" s="52">
-        <v>0.9</v>
+      <c r="F18" s="17">
+        <v>6.3</v>
       </c>
-      <c r="G18" s="52">
-        <v>-3.2</v>
+      <c r="G18" s="40">
+        <v>24.6</v>
       </c>
-      <c r="H18" s="17">
-        <v>-2.8</v>
+      <c r="H18" s="34">
+        <v>16.7</v>
       </c>
-      <c r="I18" s="40">
-        <v>21.8</v>
+      <c r="I18" s="52">
+        <v>1.7</v>
       </c>
       <c r="J18" s="34">
-        <v>16.7</v>
-      </c>
-      <c r="K18" s="52">
-        <v>1.7</v>
-      </c>
-      <c r="L18" s="34">
         <v>3.4</v>
       </c>
-      <c r="M18" s="52">
-        <v>-1.2</v>
+      <c r="K18" s="17">
+        <v>2.9</v>
       </c>
-      <c r="N18" s="52">
-        <v>-0.5</v>
-      </c>
-      <c r="O18" s="17">
-        <v>3.4</v>
-      </c>
+      <c r="L18" s="9"/>
+      <c r="M18" s="9"/>
+      <c r="N18" s="9"/>
+      <c r="O18" s="9"/>
       <c r="P18" s="9"/>
       <c r="Q18" s="9"/>
       <c r="R18" s="9"/>
       <c r="S18" s="9"/>
       <c r="T18" s="9"/>
       <c r="U18" s="9"/>
-      <c r="V18" s="9"/>
+      <c r="V18" s="12"/>
       <c r="W18" s="9"/>
       <c r="X18" s="9"/>
       <c r="Y18" s="9"/>
-      <c r="Z18" s="12"/>
+      <c r="Z18" s="9"/>
       <c r="AA18" s="9"/>
       <c r="AB18" s="9"/>
       <c r="AC18" s="9"/>
       <c r="AD18" s="9"/>
       <c r="AE18" s="9"/>
       <c r="AF18" s="9"/>
-      <c r="AG18" s="9"/>
-      <c r="AH18" s="9"/>
-      <c r="AI18" s="9"/>
-      <c r="AJ18" s="9"/>
     </row>
-    <row r="19" spans="1:36" s="10" customFormat="1">
+    <row r="19" spans="1:32" s="10" customFormat="1">
       <c r="A19" s="29" t="s">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="B19" s="14">
-        <v>38.9</v>
+        <v>47.3</v>
       </c>
       <c r="C19" s="48">
-        <v>18.2</v>
+        <v>18.3</v>
       </c>
       <c r="D19" s="14">
-        <v>13.3</v>
+        <v>9.1</v>
       </c>
       <c r="E19" s="48">
-        <v>8.1</v>
+        <v>7.3</v>
       </c>
-      <c r="F19" s="48">
-        <v>6.7</v>
+      <c r="F19" s="14">
+        <v>12.5</v>
       </c>
-      <c r="G19" s="48">
-        <v>-1.4</v>
+      <c r="G19" s="41">
+        <v>30.4</v>
       </c>
-      <c r="H19" s="14">
-        <v>7.4</v>
+      <c r="H19" s="36">
+        <v>20.3</v>
       </c>
-      <c r="I19" s="41">
-        <v>30</v>
+      <c r="I19" s="48">
+        <v>4.0999999999999996</v>
       </c>
       <c r="J19" s="36">
-        <v>20.3</v>
+        <v>5.6</v>
       </c>
-      <c r="K19" s="48">
-        <v>4.0999999999999996</v>
-      </c>
-      <c r="L19" s="36">
-        <v>3</v>
-      </c>
-      <c r="M19" s="48">
+      <c r="K19" s="14">
         <v>0.5</v>
       </c>
-      <c r="N19" s="48">
-        <v>0.6</v>
-      </c>
-      <c r="O19" s="14">
-        <v>5.6</v>
-      </c>
+      <c r="L19" s="9"/>
+      <c r="M19" s="9"/>
+      <c r="N19" s="9"/>
+      <c r="O19" s="9"/>
       <c r="P19" s="9"/>
       <c r="Q19" s="9"/>
       <c r="R19" s="9"/>
       <c r="S19" s="9"/>
       <c r="T19" s="9"/>
       <c r="U19" s="9"/>
-      <c r="V19" s="9"/>
+      <c r="V19" s="12"/>
       <c r="W19" s="9"/>
       <c r="X19" s="9"/>
       <c r="Y19" s="9"/>
-      <c r="Z19" s="12"/>
+      <c r="Z19" s="9"/>
       <c r="AA19" s="9"/>
       <c r="AB19" s="9"/>
       <c r="AC19" s="9"/>
       <c r="AD19" s="9"/>
       <c r="AE19" s="9"/>
       <c r="AF19" s="9"/>
-      <c r="AG19" s="9"/>
-      <c r="AH19" s="9"/>
-      <c r="AI19" s="9"/>
-      <c r="AJ19" s="9"/>
     </row>
-    <row r="20" spans="1:36" s="12" customFormat="1">
+    <row r="20" spans="1:32" s="12" customFormat="1">
       <c r="A20" s="29" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="B20" s="14">
-        <v>21.6</v>
+        <v>23.3</v>
       </c>
       <c r="C20" s="48">
-        <v>0.3</v>
+        <v>-0.8</v>
       </c>
       <c r="D20" s="14">
-        <v>11.1</v>
+        <v>8.1</v>
       </c>
       <c r="E20" s="48">
+        <v>9.8000000000000007</v>
+      </c>
+      <c r="F20" s="14">
+        <v>6.2</v>
+      </c>
+      <c r="G20" s="41">
+        <v>5.8</v>
+      </c>
+      <c r="H20" s="36">
         <v>3.6</v>
       </c>
-      <c r="F20" s="48">
-        <v>5.8</v>
-      </c>
-      <c r="G20" s="48">
-        <v>1.7</v>
-      </c>
-      <c r="H20" s="14">
-        <v>10.199999999999999</v>
-      </c>
-      <c r="I20" s="41">
-        <v>8.1999999999999993</v>
+      <c r="I20" s="48">
+        <v>2.4</v>
       </c>
       <c r="J20" s="36">
-        <v>3.6</v>
-      </c>
-      <c r="K20" s="48">
-        <v>2.4</v>
-      </c>
-      <c r="L20" s="36">
-        <v>-0.4</v>
-      </c>
-      <c r="M20" s="48">
-        <v>1.6</v>
-      </c>
-      <c r="N20" s="48">
-        <v>1.2</v>
-      </c>
-      <c r="O20" s="14">
         <v>2.2000000000000002</v>
       </c>
+      <c r="K20" s="14">
+        <v>-2.4</v>
+      </c>
+      <c r="L20" s="9"/>
+      <c r="M20" s="9"/>
+      <c r="N20" s="9"/>
+      <c r="O20" s="9"/>
       <c r="P20" s="9"/>
       <c r="Q20" s="9"/>
       <c r="R20" s="9"/>
       <c r="S20" s="9"/>
       <c r="T20" s="9"/>
       <c r="U20" s="9"/>
-      <c r="V20" s="9"/>
       <c r="W20" s="9"/>
       <c r="X20" s="9"/>
       <c r="Y20" s="9"/>
+      <c r="Z20" s="9"/>
       <c r="AA20" s="9"/>
       <c r="AB20" s="9"/>
       <c r="AC20" s="9"/>
       <c r="AD20" s="9"/>
       <c r="AE20" s="9"/>
       <c r="AF20" s="9"/>
-      <c r="AG20" s="9"/>
-      <c r="AH20" s="9"/>
-      <c r="AI20" s="9"/>
-      <c r="AJ20" s="9"/>
     </row>
-    <row r="21" spans="1:36" s="12" customFormat="1">
+    <row r="21" spans="1:32" s="12" customFormat="1">
       <c r="A21" s="31" t="s">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="B21" s="17">
-        <v>6.7</v>
+        <v>7.5</v>
       </c>
       <c r="C21" s="52">
         <v>-6.7</v>
@@ -20754,156 +20526,132 @@
         <v>7.3</v>
       </c>
       <c r="E21" s="52">
-        <v>-0.1</v>
-      </c>
-      <c r="F21" s="52">
-        <v>1.7</v>
-      </c>
-      <c r="G21" s="52">
-        <v>5.7</v>
-      </c>
-      <c r="H21" s="17">
         <v>6.1</v>
       </c>
-      <c r="I21" s="40">
-        <v>-10.6</v>
+      <c r="F21" s="17">
+        <v>0.8</v>
+      </c>
+      <c r="G21" s="40">
+        <v>-12.8</v>
+      </c>
+      <c r="H21" s="34">
+        <v>-5.9</v>
+      </c>
+      <c r="I21" s="52">
+        <v>-3.4</v>
       </c>
       <c r="J21" s="34">
-        <v>-5.9</v>
-      </c>
-      <c r="K21" s="52">
-        <v>-3.4</v>
-      </c>
-      <c r="L21" s="34">
-        <v>-1.9</v>
-      </c>
-      <c r="M21" s="52">
-        <v>-0.7</v>
-      </c>
-      <c r="N21" s="52">
-        <v>-0.8</v>
-      </c>
-      <c r="O21" s="17">
         <v>-1.3</v>
       </c>
+      <c r="K21" s="17">
+        <v>-2.2000000000000002</v>
+      </c>
+      <c r="L21" s="9"/>
+      <c r="M21" s="9"/>
+      <c r="N21" s="9"/>
+      <c r="O21" s="9"/>
       <c r="P21" s="9"/>
       <c r="Q21" s="9"/>
       <c r="R21" s="9"/>
       <c r="S21" s="9"/>
       <c r="T21" s="9"/>
       <c r="U21" s="9"/>
-      <c r="V21" s="9"/>
       <c r="W21" s="9"/>
       <c r="X21" s="9"/>
       <c r="Y21" s="9"/>
+      <c r="Z21" s="9"/>
       <c r="AA21" s="9"/>
       <c r="AB21" s="9"/>
       <c r="AC21" s="9"/>
       <c r="AD21" s="9"/>
       <c r="AE21" s="9"/>
       <c r="AF21" s="9"/>
-      <c r="AG21" s="9"/>
-      <c r="AH21" s="9"/>
-      <c r="AI21" s="9"/>
-      <c r="AJ21" s="9"/>
     </row>
-    <row r="22" spans="1:36" s="2" customFormat="1" ht="14.25">
+    <row r="22" spans="1:32" s="2" customFormat="1" ht="14.25">
       <c r="A22" s="30" t="s">
         <v>0</v>
       </c>
       <c r="B22" s="18">
-        <v>-9.9</v>
+        <v>-3.5</v>
       </c>
       <c r="C22" s="51">
-        <v>-1.4</v>
+        <v>-0.7</v>
       </c>
       <c r="D22" s="18">
-        <v>-10</v>
+        <v>-8.6999999999999993</v>
       </c>
       <c r="E22" s="51">
-        <v>-2.2000000000000002</v>
+        <v>2.1</v>
       </c>
-      <c r="F22" s="51">
-        <v>-5.8</v>
+      <c r="F22" s="18">
+        <v>3.8</v>
       </c>
-      <c r="G22" s="51">
-        <v>-2</v>
+      <c r="G22" s="44">
+        <v>-8.9</v>
       </c>
-      <c r="H22" s="18">
-        <v>1.5</v>
+      <c r="H22" s="39">
+        <v>-7.4</v>
       </c>
-      <c r="I22" s="44">
-        <v>-10.1</v>
+      <c r="I22" s="51">
+        <v>-3.8</v>
       </c>
       <c r="J22" s="39">
-        <v>-7.4</v>
-      </c>
-      <c r="K22" s="51">
-        <v>-3.8</v>
-      </c>
-      <c r="L22" s="39">
-        <v>-1.1000000000000001</v>
-      </c>
-      <c r="M22" s="51">
-        <v>-2.6</v>
-      </c>
-      <c r="N22" s="51">
-        <v>0</v>
-      </c>
-      <c r="O22" s="18">
         <v>1.1000000000000001</v>
       </c>
+      <c r="K22" s="18">
+        <v>1.2</v>
+      </c>
+      <c r="L22" s="9"/>
+      <c r="M22" s="9"/>
+      <c r="N22" s="9"/>
+      <c r="O22" s="9"/>
       <c r="P22" s="9"/>
       <c r="Q22" s="9"/>
       <c r="R22" s="9"/>
       <c r="S22" s="9"/>
       <c r="T22" s="9"/>
       <c r="U22" s="9"/>
-      <c r="V22" s="9"/>
       <c r="W22" s="9"/>
       <c r="X22" s="9"/>
       <c r="Y22" s="9"/>
+      <c r="Z22" s="9"/>
       <c r="AA22" s="9"/>
       <c r="AB22" s="9"/>
       <c r="AC22" s="9"/>
       <c r="AD22" s="9"/>
       <c r="AE22" s="9"/>
       <c r="AF22" s="9"/>
-      <c r="AG22" s="9"/>
-      <c r="AH22" s="9"/>
-      <c r="AI22" s="9"/>
-      <c r="AJ22" s="9"/>
     </row>
-    <row r="23" spans="1:36" ht="12.75" customHeight="1">
+    <row r="23" spans="1:32" ht="12.75" customHeight="1">
       <c r="A23" s="10"/>
+      <c r="L23" s="9"/>
+      <c r="M23" s="9"/>
+      <c r="N23" s="9"/>
+      <c r="O23" s="9"/>
       <c r="P23" s="9"/>
       <c r="Q23" s="9"/>
       <c r="R23" s="9"/>
       <c r="S23" s="9"/>
       <c r="T23" s="9"/>
-      <c r="U23" s="9"/>
-      <c r="V23" s="9"/>
-      <c r="W23" s="9"/>
-      <c r="X23" s="9"/>
-      <c r="Y23" s="12"/>
-      <c r="Z23" s="12"/>
-      <c r="AA23" s="12"/>
+      <c r="U23" s="12"/>
+      <c r="V23" s="12"/>
+      <c r="W23" s="12"/>
     </row>
-    <row r="24" spans="1:36" ht="12.75" hidden="1" customHeight="1">
-      <c r="R24" s="12"/>
+    <row r="24" spans="1:32" ht="12.75" hidden="1" customHeight="1">
+      <c r="N24" s="12"/>
+      <c r="O24" s="9"/>
+      <c r="P24" s="9"/>
+      <c r="Q24" s="9"/>
+      <c r="R24" s="9"/>
       <c r="S24" s="9"/>
       <c r="T24" s="9"/>
       <c r="U24" s="9"/>
       <c r="V24" s="9"/>
       <c r="W24" s="9"/>
-      <c r="X24" s="9"/>
-      <c r="Y24" s="9"/>
-      <c r="Z24" s="9"/>
-      <c r="AA24" s="9"/>
     </row>
-    <row r="25" spans="1:36" s="10" customFormat="1">
+    <row r="25" spans="1:32" s="10" customFormat="1">
       <c r="A25" s="11" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="12"/>
@@ -20917,14 +20665,10 @@
       <c r="K25" s="12"/>
       <c r="L25" s="12"/>
       <c r="M25" s="12"/>
-      <c r="N25" s="12"/>
-      <c r="O25" s="12"/>
-      <c r="P25" s="12"/>
-      <c r="Q25" s="12"/>
     </row>
-    <row r="26" spans="1:36" s="10" customFormat="1">
+    <row r="26" spans="1:32" s="10" customFormat="1">
       <c r="A26" s="11" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B26" s="12"/>
       <c r="C26" s="12"/>
@@ -20938,12 +20682,8 @@
       <c r="K26" s="12"/>
       <c r="L26" s="12"/>
       <c r="M26" s="12"/>
-      <c r="N26" s="12"/>
-      <c r="O26" s="12"/>
-      <c r="P26" s="12"/>
-      <c r="Q26" s="12"/>
     </row>
-    <row r="27" spans="1:36" s="10" customFormat="1">
+    <row r="27" spans="1:32" s="10" customFormat="1">
       <c r="B27" s="12"/>
       <c r="C27" s="12"/>
       <c r="D27" s="12"/>
@@ -20956,23 +20696,17 @@
       <c r="K27" s="12"/>
       <c r="L27" s="12"/>
       <c r="M27" s="12"/>
-      <c r="N27" s="12"/>
-      <c r="O27" s="12"/>
-      <c r="P27" s="12"/>
-      <c r="Q27" s="12"/>
     </row>
-    <row r="28" spans="1:36">
+    <row r="28" spans="1:32">
       <c r="A28" s="8" t="s">
-        <v>34</v>
+        <v>21</v>
       </c>
     </row>
-    <row r="31" spans="1:36">
+    <row r="31" spans="1:32">
       <c r="A31" s="5"/>
     </row>
   </sheetData>
-  <mergeCells count="8">
-    <mergeCell ref="H4:H5"/>
-    <mergeCell ref="G4:G5"/>
+  <mergeCells count="6">
     <mergeCell ref="F4:F5"/>
     <mergeCell ref="E4:E5"/>
     <mergeCell ref="A4:A5"/>
@@ -21220,16 +20954,16 @@
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6839A8CB-A185-4F2B-8CCC-C75CA1978D0E}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="fa7ed35a-250d-45d0-9580-0207d5f6dcb4"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="fa7ed35a-250d-45d0-9580-0207d5f6dcb4"/>
     <ds:schemaRef ds:uri="132f1bae-ffcd-44c6-a909-953ed45d18e3"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>